<commit_message>
feat: Implement 22-Point Daily Genset Checklist with side-by-side tick checkboxes
</commit_message>
<xml_diff>
--- a/genset_readings.xlsx
+++ b/genset_readings.xlsx
@@ -1256,7 +1256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U35"/>
+  <dimension ref="A1:AS35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -1268,6 +1268,30 @@
     <col width="13" customWidth="1" min="19" max="19"/>
     <col width="13" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="13" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="31" max="31"/>
+    <col width="13" customWidth="1" min="32" max="32"/>
+    <col width="13" customWidth="1" min="33" max="33"/>
+    <col width="13" customWidth="1" min="34" max="34"/>
+    <col width="13" customWidth="1" min="35" max="35"/>
+    <col width="13" customWidth="1" min="36" max="36"/>
+    <col width="13" customWidth="1" min="37" max="37"/>
+    <col width="13" customWidth="1" min="38" max="38"/>
+    <col width="13" customWidth="1" min="39" max="39"/>
+    <col width="13" customWidth="1" min="40" max="40"/>
+    <col width="13" customWidth="1" min="41" max="41"/>
+    <col width="13" customWidth="1" min="42" max="42"/>
+    <col width="13" customWidth="1" min="43" max="43"/>
+    <col width="13" customWidth="1" min="44" max="44"/>
+    <col width="13" customWidth="1" min="45" max="45"/>
   </cols>
   <sheetData>
     <row r="1" ht="32.25" customHeight="1">
@@ -1293,20 +1317,44 @@
       <c r="P1" s="23" t="n"/>
       <c r="Q1" s="23" t="n"/>
       <c r="R1" s="23" t="n"/>
-      <c r="S1" s="24" t="n"/>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="S1" s="23" t="n"/>
+      <c r="T1" s="23" t="n"/>
+      <c r="U1" s="23" t="n"/>
+      <c r="V1" s="23" t="n"/>
+      <c r="W1" s="23" t="n"/>
+      <c r="X1" s="23" t="n"/>
+      <c r="Y1" s="23" t="n"/>
+      <c r="Z1" s="23" t="n"/>
+      <c r="AA1" s="23" t="n"/>
+      <c r="AB1" s="23" t="n"/>
+      <c r="AC1" s="23" t="n"/>
+      <c r="AD1" s="23" t="n"/>
+      <c r="AE1" s="23" t="n"/>
+      <c r="AF1" s="23" t="n"/>
+      <c r="AG1" s="23" t="n"/>
+      <c r="AH1" s="23" t="n"/>
+      <c r="AI1" s="23" t="n"/>
+      <c r="AJ1" s="23" t="n"/>
+      <c r="AK1" s="23" t="n"/>
+      <c r="AL1" s="23" t="n"/>
+      <c r="AM1" s="23" t="n"/>
+      <c r="AN1" s="23" t="n"/>
+      <c r="AO1" s="23" t="n"/>
+      <c r="AP1" s="24" t="n"/>
+      <c r="AQ1" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DOC NO: R/MAI/GS
 MONTH/YEAR: </t>
         </is>
       </c>
-      <c r="U1" s="24" t="n"/>
+      <c r="AR1" s="23" t="n"/>
+      <c r="AS1" s="24" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="6" t="n"/>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>DAILY GENSET CHECKLIST</t>
+          <t>22-POINT DAILY GENSET CHECKLIST</t>
         </is>
       </c>
       <c r="C2" s="25" t="n"/>
@@ -1327,7 +1375,31 @@
       <c r="R2" s="25" t="n"/>
       <c r="S2" s="25" t="n"/>
       <c r="T2" s="25" t="n"/>
-      <c r="U2" s="26" t="n"/>
+      <c r="U2" s="25" t="n"/>
+      <c r="V2" s="25" t="n"/>
+      <c r="W2" s="25" t="n"/>
+      <c r="X2" s="25" t="n"/>
+      <c r="Y2" s="25" t="n"/>
+      <c r="Z2" s="25" t="n"/>
+      <c r="AA2" s="25" t="n"/>
+      <c r="AB2" s="25" t="n"/>
+      <c r="AC2" s="25" t="n"/>
+      <c r="AD2" s="25" t="n"/>
+      <c r="AE2" s="25" t="n"/>
+      <c r="AF2" s="25" t="n"/>
+      <c r="AG2" s="25" t="n"/>
+      <c r="AH2" s="25" t="n"/>
+      <c r="AI2" s="25" t="n"/>
+      <c r="AJ2" s="25" t="n"/>
+      <c r="AK2" s="25" t="n"/>
+      <c r="AL2" s="25" t="n"/>
+      <c r="AM2" s="25" t="n"/>
+      <c r="AN2" s="25" t="n"/>
+      <c r="AO2" s="25" t="n"/>
+      <c r="AP2" s="25" t="n"/>
+      <c r="AQ2" s="25" t="n"/>
+      <c r="AR2" s="25" t="n"/>
+      <c r="AS2" s="26" t="n"/>
     </row>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -1337,102 +1409,222 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>G1 MODE</t>
+          <t>G1 Q1</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>G1 RUN HRS</t>
+          <t>G1 Q2</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>G1 BATT VOLT</t>
+          <t>G1 Q3</t>
         </is>
       </c>
       <c r="E3" s="10" t="inlineStr">
         <is>
-          <t>G1 LUBE OIL</t>
+          <t>G1 Q4</t>
         </is>
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>G1 COOLANT</t>
+          <t>G1 Q5</t>
         </is>
       </c>
       <c r="G3" s="10" t="inlineStr">
         <is>
-          <t>G1 FUEL %</t>
+          <t>G1 Q6</t>
         </is>
       </c>
       <c r="H3" s="10" t="inlineStr">
         <is>
-          <t>G1 VOLT R</t>
+          <t>G1 Q7</t>
         </is>
       </c>
       <c r="I3" s="10" t="inlineStr">
         <is>
-          <t>G1 VOLT Y</t>
+          <t>G1 Q8</t>
         </is>
       </c>
       <c r="J3" s="10" t="inlineStr">
         <is>
-          <t>G1 VOLT B</t>
+          <t>G1 Q9</t>
         </is>
       </c>
       <c r="K3" s="10" t="inlineStr">
         <is>
-          <t>G1 FREQ</t>
+          <t>G1 Q10</t>
         </is>
       </c>
       <c r="L3" s="10" t="inlineStr">
         <is>
-          <t>G2 MODE</t>
+          <t>G1 Q11</t>
         </is>
       </c>
       <c r="M3" s="11" t="inlineStr">
         <is>
-          <t>G2 RUN HRS</t>
+          <t>G1 Q12</t>
         </is>
       </c>
       <c r="N3" s="10" t="inlineStr">
         <is>
-          <t>G2 BATT VOLT</t>
+          <t>G1 Q13</t>
         </is>
       </c>
       <c r="O3" s="10" t="inlineStr">
         <is>
-          <t>G2 LUBE OIL</t>
+          <t>G1 Q14</t>
         </is>
       </c>
       <c r="P3" s="10" t="inlineStr">
         <is>
-          <t>G2 COOLANT</t>
+          <t>G1 Q15</t>
         </is>
       </c>
       <c r="Q3" s="10" t="inlineStr">
         <is>
-          <t>G2 FUEL %</t>
+          <t>G1 Q16</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
         <is>
-          <t>G2 VOLT R</t>
+          <t>G1 Q17</t>
         </is>
       </c>
       <c r="S3" s="10" t="inlineStr">
         <is>
-          <t>G2 VOLT Y</t>
+          <t>G1 Q18</t>
         </is>
       </c>
       <c r="T3" s="10" t="inlineStr">
         <is>
-          <t>G2 VOLT B</t>
+          <t>G1 Q19</t>
         </is>
       </c>
       <c r="U3" s="10" t="inlineStr">
         <is>
-          <t>G2 FREQ</t>
+          <t>G1 Q20</t>
+        </is>
+      </c>
+      <c r="V3" s="10" t="inlineStr">
+        <is>
+          <t>G1 Q21</t>
+        </is>
+      </c>
+      <c r="W3" s="10" t="inlineStr">
+        <is>
+          <t>G1 Q22</t>
+        </is>
+      </c>
+      <c r="X3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q1</t>
+        </is>
+      </c>
+      <c r="Y3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q2</t>
+        </is>
+      </c>
+      <c r="Z3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q3</t>
+        </is>
+      </c>
+      <c r="AA3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q4</t>
+        </is>
+      </c>
+      <c r="AB3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q5</t>
+        </is>
+      </c>
+      <c r="AC3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q6</t>
+        </is>
+      </c>
+      <c r="AD3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q7</t>
+        </is>
+      </c>
+      <c r="AE3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q8</t>
+        </is>
+      </c>
+      <c r="AF3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q9</t>
+        </is>
+      </c>
+      <c r="AG3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q10</t>
+        </is>
+      </c>
+      <c r="AH3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q11</t>
+        </is>
+      </c>
+      <c r="AI3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q12</t>
+        </is>
+      </c>
+      <c r="AJ3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q13</t>
+        </is>
+      </c>
+      <c r="AK3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q14</t>
+        </is>
+      </c>
+      <c r="AL3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q15</t>
+        </is>
+      </c>
+      <c r="AM3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q16</t>
+        </is>
+      </c>
+      <c r="AN3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q17</t>
+        </is>
+      </c>
+      <c r="AO3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q18</t>
+        </is>
+      </c>
+      <c r="AP3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q19</t>
+        </is>
+      </c>
+      <c r="AQ3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q20</t>
+        </is>
+      </c>
+      <c r="AR3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q21</t>
+        </is>
+      </c>
+      <c r="AS3" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q22</t>
         </is>
       </c>
     </row>
@@ -1460,6 +1652,30 @@
       <c r="S4" s="27" t="n"/>
       <c r="T4" s="27" t="n"/>
       <c r="U4" s="27" t="n"/>
+      <c r="V4" s="27" t="n"/>
+      <c r="W4" s="27" t="n"/>
+      <c r="X4" s="27" t="n"/>
+      <c r="Y4" s="27" t="n"/>
+      <c r="Z4" s="27" t="n"/>
+      <c r="AA4" s="27" t="n"/>
+      <c r="AB4" s="27" t="n"/>
+      <c r="AC4" s="27" t="n"/>
+      <c r="AD4" s="27" t="n"/>
+      <c r="AE4" s="27" t="n"/>
+      <c r="AF4" s="27" t="n"/>
+      <c r="AG4" s="27" t="n"/>
+      <c r="AH4" s="27" t="n"/>
+      <c r="AI4" s="27" t="n"/>
+      <c r="AJ4" s="27" t="n"/>
+      <c r="AK4" s="27" t="n"/>
+      <c r="AL4" s="27" t="n"/>
+      <c r="AM4" s="27" t="n"/>
+      <c r="AN4" s="27" t="n"/>
+      <c r="AO4" s="27" t="n"/>
+      <c r="AP4" s="27" t="n"/>
+      <c r="AQ4" s="27" t="n"/>
+      <c r="AR4" s="27" t="n"/>
+      <c r="AS4" s="27" t="n"/>
     </row>
     <row r="5" ht="33" customHeight="1">
       <c r="A5" s="12" t="n">
@@ -1485,6 +1701,30 @@
       <c r="S5" s="27" t="n"/>
       <c r="T5" s="27" t="n"/>
       <c r="U5" s="27" t="n"/>
+      <c r="V5" s="27" t="n"/>
+      <c r="W5" s="27" t="n"/>
+      <c r="X5" s="27" t="n"/>
+      <c r="Y5" s="27" t="n"/>
+      <c r="Z5" s="27" t="n"/>
+      <c r="AA5" s="27" t="n"/>
+      <c r="AB5" s="27" t="n"/>
+      <c r="AC5" s="27" t="n"/>
+      <c r="AD5" s="27" t="n"/>
+      <c r="AE5" s="27" t="n"/>
+      <c r="AF5" s="27" t="n"/>
+      <c r="AG5" s="27" t="n"/>
+      <c r="AH5" s="27" t="n"/>
+      <c r="AI5" s="27" t="n"/>
+      <c r="AJ5" s="27" t="n"/>
+      <c r="AK5" s="27" t="n"/>
+      <c r="AL5" s="27" t="n"/>
+      <c r="AM5" s="27" t="n"/>
+      <c r="AN5" s="27" t="n"/>
+      <c r="AO5" s="27" t="n"/>
+      <c r="AP5" s="27" t="n"/>
+      <c r="AQ5" s="27" t="n"/>
+      <c r="AR5" s="27" t="n"/>
+      <c r="AS5" s="27" t="n"/>
     </row>
     <row r="6" ht="33" customHeight="1">
       <c r="A6" s="12" t="n">
@@ -1510,6 +1750,30 @@
       <c r="S6" s="27" t="n"/>
       <c r="T6" s="27" t="n"/>
       <c r="U6" s="27" t="n"/>
+      <c r="V6" s="27" t="n"/>
+      <c r="W6" s="27" t="n"/>
+      <c r="X6" s="27" t="n"/>
+      <c r="Y6" s="27" t="n"/>
+      <c r="Z6" s="27" t="n"/>
+      <c r="AA6" s="27" t="n"/>
+      <c r="AB6" s="27" t="n"/>
+      <c r="AC6" s="27" t="n"/>
+      <c r="AD6" s="27" t="n"/>
+      <c r="AE6" s="27" t="n"/>
+      <c r="AF6" s="27" t="n"/>
+      <c r="AG6" s="27" t="n"/>
+      <c r="AH6" s="27" t="n"/>
+      <c r="AI6" s="27" t="n"/>
+      <c r="AJ6" s="27" t="n"/>
+      <c r="AK6" s="27" t="n"/>
+      <c r="AL6" s="27" t="n"/>
+      <c r="AM6" s="27" t="n"/>
+      <c r="AN6" s="27" t="n"/>
+      <c r="AO6" s="27" t="n"/>
+      <c r="AP6" s="27" t="n"/>
+      <c r="AQ6" s="27" t="n"/>
+      <c r="AR6" s="27" t="n"/>
+      <c r="AS6" s="27" t="n"/>
     </row>
     <row r="7" ht="33" customHeight="1">
       <c r="A7" s="12" t="n">
@@ -1535,6 +1799,30 @@
       <c r="S7" s="27" t="n"/>
       <c r="T7" s="27" t="n"/>
       <c r="U7" s="27" t="n"/>
+      <c r="V7" s="27" t="n"/>
+      <c r="W7" s="27" t="n"/>
+      <c r="X7" s="27" t="n"/>
+      <c r="Y7" s="27" t="n"/>
+      <c r="Z7" s="27" t="n"/>
+      <c r="AA7" s="27" t="n"/>
+      <c r="AB7" s="27" t="n"/>
+      <c r="AC7" s="27" t="n"/>
+      <c r="AD7" s="27" t="n"/>
+      <c r="AE7" s="27" t="n"/>
+      <c r="AF7" s="27" t="n"/>
+      <c r="AG7" s="27" t="n"/>
+      <c r="AH7" s="27" t="n"/>
+      <c r="AI7" s="27" t="n"/>
+      <c r="AJ7" s="27" t="n"/>
+      <c r="AK7" s="27" t="n"/>
+      <c r="AL7" s="27" t="n"/>
+      <c r="AM7" s="27" t="n"/>
+      <c r="AN7" s="27" t="n"/>
+      <c r="AO7" s="27" t="n"/>
+      <c r="AP7" s="27" t="n"/>
+      <c r="AQ7" s="27" t="n"/>
+      <c r="AR7" s="27" t="n"/>
+      <c r="AS7" s="27" t="n"/>
     </row>
     <row r="8" ht="33" customHeight="1">
       <c r="A8" s="12" t="n">
@@ -1560,6 +1848,30 @@
       <c r="S8" s="27" t="n"/>
       <c r="T8" s="27" t="n"/>
       <c r="U8" s="27" t="n"/>
+      <c r="V8" s="27" t="n"/>
+      <c r="W8" s="27" t="n"/>
+      <c r="X8" s="27" t="n"/>
+      <c r="Y8" s="27" t="n"/>
+      <c r="Z8" s="27" t="n"/>
+      <c r="AA8" s="27" t="n"/>
+      <c r="AB8" s="27" t="n"/>
+      <c r="AC8" s="27" t="n"/>
+      <c r="AD8" s="27" t="n"/>
+      <c r="AE8" s="27" t="n"/>
+      <c r="AF8" s="27" t="n"/>
+      <c r="AG8" s="27" t="n"/>
+      <c r="AH8" s="27" t="n"/>
+      <c r="AI8" s="27" t="n"/>
+      <c r="AJ8" s="27" t="n"/>
+      <c r="AK8" s="27" t="n"/>
+      <c r="AL8" s="27" t="n"/>
+      <c r="AM8" s="27" t="n"/>
+      <c r="AN8" s="27" t="n"/>
+      <c r="AO8" s="27" t="n"/>
+      <c r="AP8" s="27" t="n"/>
+      <c r="AQ8" s="27" t="n"/>
+      <c r="AR8" s="27" t="n"/>
+      <c r="AS8" s="27" t="n"/>
     </row>
     <row r="9" ht="33" customHeight="1">
       <c r="A9" s="12" t="n">
@@ -1585,6 +1897,30 @@
       <c r="S9" s="27" t="n"/>
       <c r="T9" s="27" t="n"/>
       <c r="U9" s="27" t="n"/>
+      <c r="V9" s="27" t="n"/>
+      <c r="W9" s="27" t="n"/>
+      <c r="X9" s="27" t="n"/>
+      <c r="Y9" s="27" t="n"/>
+      <c r="Z9" s="27" t="n"/>
+      <c r="AA9" s="27" t="n"/>
+      <c r="AB9" s="27" t="n"/>
+      <c r="AC9" s="27" t="n"/>
+      <c r="AD9" s="27" t="n"/>
+      <c r="AE9" s="27" t="n"/>
+      <c r="AF9" s="27" t="n"/>
+      <c r="AG9" s="27" t="n"/>
+      <c r="AH9" s="27" t="n"/>
+      <c r="AI9" s="27" t="n"/>
+      <c r="AJ9" s="27" t="n"/>
+      <c r="AK9" s="27" t="n"/>
+      <c r="AL9" s="27" t="n"/>
+      <c r="AM9" s="27" t="n"/>
+      <c r="AN9" s="27" t="n"/>
+      <c r="AO9" s="27" t="n"/>
+      <c r="AP9" s="27" t="n"/>
+      <c r="AQ9" s="27" t="n"/>
+      <c r="AR9" s="27" t="n"/>
+      <c r="AS9" s="27" t="n"/>
     </row>
     <row r="10" ht="33" customHeight="1">
       <c r="A10" s="15" t="n">
@@ -1610,6 +1946,30 @@
       <c r="S10" s="28" t="n"/>
       <c r="T10" s="28" t="n"/>
       <c r="U10" s="28" t="n"/>
+      <c r="V10" s="28" t="n"/>
+      <c r="W10" s="28" t="n"/>
+      <c r="X10" s="28" t="n"/>
+      <c r="Y10" s="28" t="n"/>
+      <c r="Z10" s="28" t="n"/>
+      <c r="AA10" s="28" t="n"/>
+      <c r="AB10" s="28" t="n"/>
+      <c r="AC10" s="28" t="n"/>
+      <c r="AD10" s="28" t="n"/>
+      <c r="AE10" s="28" t="n"/>
+      <c r="AF10" s="28" t="n"/>
+      <c r="AG10" s="28" t="n"/>
+      <c r="AH10" s="28" t="n"/>
+      <c r="AI10" s="28" t="n"/>
+      <c r="AJ10" s="28" t="n"/>
+      <c r="AK10" s="28" t="n"/>
+      <c r="AL10" s="28" t="n"/>
+      <c r="AM10" s="28" t="n"/>
+      <c r="AN10" s="28" t="n"/>
+      <c r="AO10" s="28" t="n"/>
+      <c r="AP10" s="28" t="n"/>
+      <c r="AQ10" s="28" t="n"/>
+      <c r="AR10" s="28" t="n"/>
+      <c r="AS10" s="28" t="n"/>
     </row>
     <row r="11" ht="33" customHeight="1">
       <c r="A11" s="12" t="n">
@@ -1635,6 +1995,30 @@
       <c r="S11" s="27" t="n"/>
       <c r="T11" s="27" t="n"/>
       <c r="U11" s="27" t="n"/>
+      <c r="V11" s="27" t="n"/>
+      <c r="W11" s="27" t="n"/>
+      <c r="X11" s="27" t="n"/>
+      <c r="Y11" s="27" t="n"/>
+      <c r="Z11" s="27" t="n"/>
+      <c r="AA11" s="27" t="n"/>
+      <c r="AB11" s="27" t="n"/>
+      <c r="AC11" s="27" t="n"/>
+      <c r="AD11" s="27" t="n"/>
+      <c r="AE11" s="27" t="n"/>
+      <c r="AF11" s="27" t="n"/>
+      <c r="AG11" s="27" t="n"/>
+      <c r="AH11" s="27" t="n"/>
+      <c r="AI11" s="27" t="n"/>
+      <c r="AJ11" s="27" t="n"/>
+      <c r="AK11" s="27" t="n"/>
+      <c r="AL11" s="27" t="n"/>
+      <c r="AM11" s="27" t="n"/>
+      <c r="AN11" s="27" t="n"/>
+      <c r="AO11" s="27" t="n"/>
+      <c r="AP11" s="27" t="n"/>
+      <c r="AQ11" s="27" t="n"/>
+      <c r="AR11" s="27" t="n"/>
+      <c r="AS11" s="27" t="n"/>
     </row>
     <row r="12" ht="33" customHeight="1">
       <c r="A12" s="12" t="n">
@@ -1660,6 +2044,30 @@
       <c r="S12" s="27" t="n"/>
       <c r="T12" s="27" t="n"/>
       <c r="U12" s="27" t="n"/>
+      <c r="V12" s="27" t="n"/>
+      <c r="W12" s="27" t="n"/>
+      <c r="X12" s="27" t="n"/>
+      <c r="Y12" s="27" t="n"/>
+      <c r="Z12" s="27" t="n"/>
+      <c r="AA12" s="27" t="n"/>
+      <c r="AB12" s="27" t="n"/>
+      <c r="AC12" s="27" t="n"/>
+      <c r="AD12" s="27" t="n"/>
+      <c r="AE12" s="27" t="n"/>
+      <c r="AF12" s="27" t="n"/>
+      <c r="AG12" s="27" t="n"/>
+      <c r="AH12" s="27" t="n"/>
+      <c r="AI12" s="27" t="n"/>
+      <c r="AJ12" s="27" t="n"/>
+      <c r="AK12" s="27" t="n"/>
+      <c r="AL12" s="27" t="n"/>
+      <c r="AM12" s="27" t="n"/>
+      <c r="AN12" s="27" t="n"/>
+      <c r="AO12" s="27" t="n"/>
+      <c r="AP12" s="27" t="n"/>
+      <c r="AQ12" s="27" t="n"/>
+      <c r="AR12" s="27" t="n"/>
+      <c r="AS12" s="27" t="n"/>
     </row>
     <row r="13" ht="33" customHeight="1">
       <c r="A13" s="12" t="n">
@@ -1685,6 +2093,30 @@
       <c r="S13" s="27" t="n"/>
       <c r="T13" s="27" t="n"/>
       <c r="U13" s="27" t="n"/>
+      <c r="V13" s="27" t="n"/>
+      <c r="W13" s="27" t="n"/>
+      <c r="X13" s="27" t="n"/>
+      <c r="Y13" s="27" t="n"/>
+      <c r="Z13" s="27" t="n"/>
+      <c r="AA13" s="27" t="n"/>
+      <c r="AB13" s="27" t="n"/>
+      <c r="AC13" s="27" t="n"/>
+      <c r="AD13" s="27" t="n"/>
+      <c r="AE13" s="27" t="n"/>
+      <c r="AF13" s="27" t="n"/>
+      <c r="AG13" s="27" t="n"/>
+      <c r="AH13" s="27" t="n"/>
+      <c r="AI13" s="27" t="n"/>
+      <c r="AJ13" s="27" t="n"/>
+      <c r="AK13" s="27" t="n"/>
+      <c r="AL13" s="27" t="n"/>
+      <c r="AM13" s="27" t="n"/>
+      <c r="AN13" s="27" t="n"/>
+      <c r="AO13" s="27" t="n"/>
+      <c r="AP13" s="27" t="n"/>
+      <c r="AQ13" s="27" t="n"/>
+      <c r="AR13" s="27" t="n"/>
+      <c r="AS13" s="27" t="n"/>
     </row>
     <row r="14" ht="33" customHeight="1">
       <c r="A14" s="12" t="n">
@@ -1710,6 +2142,30 @@
       <c r="S14" s="27" t="n"/>
       <c r="T14" s="27" t="n"/>
       <c r="U14" s="27" t="n"/>
+      <c r="V14" s="27" t="n"/>
+      <c r="W14" s="27" t="n"/>
+      <c r="X14" s="27" t="n"/>
+      <c r="Y14" s="27" t="n"/>
+      <c r="Z14" s="27" t="n"/>
+      <c r="AA14" s="27" t="n"/>
+      <c r="AB14" s="27" t="n"/>
+      <c r="AC14" s="27" t="n"/>
+      <c r="AD14" s="27" t="n"/>
+      <c r="AE14" s="27" t="n"/>
+      <c r="AF14" s="27" t="n"/>
+      <c r="AG14" s="27" t="n"/>
+      <c r="AH14" s="27" t="n"/>
+      <c r="AI14" s="27" t="n"/>
+      <c r="AJ14" s="27" t="n"/>
+      <c r="AK14" s="27" t="n"/>
+      <c r="AL14" s="27" t="n"/>
+      <c r="AM14" s="27" t="n"/>
+      <c r="AN14" s="27" t="n"/>
+      <c r="AO14" s="27" t="n"/>
+      <c r="AP14" s="27" t="n"/>
+      <c r="AQ14" s="27" t="n"/>
+      <c r="AR14" s="27" t="n"/>
+      <c r="AS14" s="27" t="n"/>
     </row>
     <row r="15" ht="33" customHeight="1">
       <c r="A15" s="12" t="n">
@@ -1735,6 +2191,30 @@
       <c r="S15" s="27" t="n"/>
       <c r="T15" s="27" t="n"/>
       <c r="U15" s="27" t="n"/>
+      <c r="V15" s="27" t="n"/>
+      <c r="W15" s="27" t="n"/>
+      <c r="X15" s="27" t="n"/>
+      <c r="Y15" s="27" t="n"/>
+      <c r="Z15" s="27" t="n"/>
+      <c r="AA15" s="27" t="n"/>
+      <c r="AB15" s="27" t="n"/>
+      <c r="AC15" s="27" t="n"/>
+      <c r="AD15" s="27" t="n"/>
+      <c r="AE15" s="27" t="n"/>
+      <c r="AF15" s="27" t="n"/>
+      <c r="AG15" s="27" t="n"/>
+      <c r="AH15" s="27" t="n"/>
+      <c r="AI15" s="27" t="n"/>
+      <c r="AJ15" s="27" t="n"/>
+      <c r="AK15" s="27" t="n"/>
+      <c r="AL15" s="27" t="n"/>
+      <c r="AM15" s="27" t="n"/>
+      <c r="AN15" s="27" t="n"/>
+      <c r="AO15" s="27" t="n"/>
+      <c r="AP15" s="27" t="n"/>
+      <c r="AQ15" s="27" t="n"/>
+      <c r="AR15" s="27" t="n"/>
+      <c r="AS15" s="27" t="n"/>
     </row>
     <row r="16" ht="33" customHeight="1">
       <c r="A16" s="12" t="n">
@@ -1760,6 +2240,30 @@
       <c r="S16" s="27" t="n"/>
       <c r="T16" s="27" t="n"/>
       <c r="U16" s="27" t="n"/>
+      <c r="V16" s="27" t="n"/>
+      <c r="W16" s="27" t="n"/>
+      <c r="X16" s="27" t="n"/>
+      <c r="Y16" s="27" t="n"/>
+      <c r="Z16" s="27" t="n"/>
+      <c r="AA16" s="27" t="n"/>
+      <c r="AB16" s="27" t="n"/>
+      <c r="AC16" s="27" t="n"/>
+      <c r="AD16" s="27" t="n"/>
+      <c r="AE16" s="27" t="n"/>
+      <c r="AF16" s="27" t="n"/>
+      <c r="AG16" s="27" t="n"/>
+      <c r="AH16" s="27" t="n"/>
+      <c r="AI16" s="27" t="n"/>
+      <c r="AJ16" s="27" t="n"/>
+      <c r="AK16" s="27" t="n"/>
+      <c r="AL16" s="27" t="n"/>
+      <c r="AM16" s="27" t="n"/>
+      <c r="AN16" s="27" t="n"/>
+      <c r="AO16" s="27" t="n"/>
+      <c r="AP16" s="27" t="n"/>
+      <c r="AQ16" s="27" t="n"/>
+      <c r="AR16" s="27" t="n"/>
+      <c r="AS16" s="27" t="n"/>
     </row>
     <row r="17" ht="33" customHeight="1">
       <c r="A17" s="15" t="n">
@@ -1785,6 +2289,30 @@
       <c r="S17" s="28" t="n"/>
       <c r="T17" s="28" t="n"/>
       <c r="U17" s="28" t="n"/>
+      <c r="V17" s="28" t="n"/>
+      <c r="W17" s="28" t="n"/>
+      <c r="X17" s="28" t="n"/>
+      <c r="Y17" s="28" t="n"/>
+      <c r="Z17" s="28" t="n"/>
+      <c r="AA17" s="28" t="n"/>
+      <c r="AB17" s="28" t="n"/>
+      <c r="AC17" s="28" t="n"/>
+      <c r="AD17" s="28" t="n"/>
+      <c r="AE17" s="28" t="n"/>
+      <c r="AF17" s="28" t="n"/>
+      <c r="AG17" s="28" t="n"/>
+      <c r="AH17" s="28" t="n"/>
+      <c r="AI17" s="28" t="n"/>
+      <c r="AJ17" s="28" t="n"/>
+      <c r="AK17" s="28" t="n"/>
+      <c r="AL17" s="28" t="n"/>
+      <c r="AM17" s="28" t="n"/>
+      <c r="AN17" s="28" t="n"/>
+      <c r="AO17" s="28" t="n"/>
+      <c r="AP17" s="28" t="n"/>
+      <c r="AQ17" s="28" t="n"/>
+      <c r="AR17" s="28" t="n"/>
+      <c r="AS17" s="28" t="n"/>
     </row>
     <row r="18" ht="33" customHeight="1">
       <c r="A18" s="12" t="n">
@@ -1810,12 +2338,36 @@
       <c r="S18" s="27" t="n"/>
       <c r="T18" s="27" t="n"/>
       <c r="U18" s="27" t="n"/>
+      <c r="V18" s="27" t="n"/>
+      <c r="W18" s="27" t="n"/>
+      <c r="X18" s="27" t="n"/>
+      <c r="Y18" s="27" t="n"/>
+      <c r="Z18" s="27" t="n"/>
+      <c r="AA18" s="27" t="n"/>
+      <c r="AB18" s="27" t="n"/>
+      <c r="AC18" s="27" t="n"/>
+      <c r="AD18" s="27" t="n"/>
+      <c r="AE18" s="27" t="n"/>
+      <c r="AF18" s="27" t="n"/>
+      <c r="AG18" s="27" t="n"/>
+      <c r="AH18" s="27" t="n"/>
+      <c r="AI18" s="27" t="n"/>
+      <c r="AJ18" s="27" t="n"/>
+      <c r="AK18" s="27" t="n"/>
+      <c r="AL18" s="27" t="n"/>
+      <c r="AM18" s="27" t="n"/>
+      <c r="AN18" s="27" t="n"/>
+      <c r="AO18" s="27" t="n"/>
+      <c r="AP18" s="27" t="n"/>
+      <c r="AQ18" s="27" t="n"/>
+      <c r="AR18" s="27" t="n"/>
+      <c r="AS18" s="27" t="n"/>
     </row>
     <row r="19" ht="33" customHeight="1">
       <c r="A19" s="6" t="n"/>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>DAILY GENSET CHECKLIST</t>
+          <t>22-POINT DAILY GENSET CHECKLIST</t>
         </is>
       </c>
       <c r="C19" s="25" t="n"/>
@@ -1836,7 +2388,31 @@
       <c r="R19" s="25" t="n"/>
       <c r="S19" s="25" t="n"/>
       <c r="T19" s="25" t="n"/>
-      <c r="U19" s="26" t="n"/>
+      <c r="U19" s="25" t="n"/>
+      <c r="V19" s="25" t="n"/>
+      <c r="W19" s="25" t="n"/>
+      <c r="X19" s="25" t="n"/>
+      <c r="Y19" s="25" t="n"/>
+      <c r="Z19" s="25" t="n"/>
+      <c r="AA19" s="25" t="n"/>
+      <c r="AB19" s="25" t="n"/>
+      <c r="AC19" s="25" t="n"/>
+      <c r="AD19" s="25" t="n"/>
+      <c r="AE19" s="25" t="n"/>
+      <c r="AF19" s="25" t="n"/>
+      <c r="AG19" s="25" t="n"/>
+      <c r="AH19" s="25" t="n"/>
+      <c r="AI19" s="25" t="n"/>
+      <c r="AJ19" s="25" t="n"/>
+      <c r="AK19" s="25" t="n"/>
+      <c r="AL19" s="25" t="n"/>
+      <c r="AM19" s="25" t="n"/>
+      <c r="AN19" s="25" t="n"/>
+      <c r="AO19" s="25" t="n"/>
+      <c r="AP19" s="25" t="n"/>
+      <c r="AQ19" s="25" t="n"/>
+      <c r="AR19" s="25" t="n"/>
+      <c r="AS19" s="26" t="n"/>
     </row>
     <row r="20" ht="59.25" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
@@ -1846,102 +2422,222 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>G1 MODE</t>
+          <t>G1 Q1</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>G1 RUN HRS</t>
+          <t>G1 Q2</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>G1 BATT VOLT</t>
+          <t>G1 Q3</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>G1 LUBE OIL</t>
+          <t>G1 Q4</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>G1 COOLANT</t>
+          <t>G1 Q5</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>G1 FUEL %</t>
+          <t>G1 Q6</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>G1 VOLT R</t>
+          <t>G1 Q7</t>
         </is>
       </c>
       <c r="I20" s="10" t="inlineStr">
         <is>
-          <t>G1 VOLT Y</t>
+          <t>G1 Q8</t>
         </is>
       </c>
       <c r="J20" s="10" t="inlineStr">
         <is>
-          <t>G1 VOLT B</t>
+          <t>G1 Q9</t>
         </is>
       </c>
       <c r="K20" s="10" t="inlineStr">
         <is>
-          <t>G1 FREQ</t>
+          <t>G1 Q10</t>
         </is>
       </c>
       <c r="L20" s="10" t="inlineStr">
         <is>
-          <t>G2 MODE</t>
+          <t>G1 Q11</t>
         </is>
       </c>
       <c r="M20" s="11" t="inlineStr">
         <is>
-          <t>G2 RUN HRS</t>
+          <t>G1 Q12</t>
         </is>
       </c>
       <c r="N20" s="10" t="inlineStr">
         <is>
-          <t>G2 BATT VOLT</t>
+          <t>G1 Q13</t>
         </is>
       </c>
       <c r="O20" s="10" t="inlineStr">
         <is>
-          <t>G2 LUBE OIL</t>
+          <t>G1 Q14</t>
         </is>
       </c>
       <c r="P20" s="10" t="inlineStr">
         <is>
-          <t>G2 COOLANT</t>
+          <t>G1 Q15</t>
         </is>
       </c>
       <c r="Q20" s="10" t="inlineStr">
         <is>
-          <t>G2 FUEL %</t>
+          <t>G1 Q16</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
         <is>
-          <t>G2 VOLT R</t>
+          <t>G1 Q17</t>
         </is>
       </c>
       <c r="S20" s="10" t="inlineStr">
         <is>
-          <t>G2 VOLT Y</t>
+          <t>G1 Q18</t>
         </is>
       </c>
       <c r="T20" s="10" t="inlineStr">
         <is>
-          <t>G2 VOLT B</t>
+          <t>G1 Q19</t>
         </is>
       </c>
       <c r="U20" s="10" t="inlineStr">
         <is>
-          <t>G2 FREQ</t>
+          <t>G1 Q20</t>
+        </is>
+      </c>
+      <c r="V20" s="10" t="inlineStr">
+        <is>
+          <t>G1 Q21</t>
+        </is>
+      </c>
+      <c r="W20" s="10" t="inlineStr">
+        <is>
+          <t>G1 Q22</t>
+        </is>
+      </c>
+      <c r="X20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q1</t>
+        </is>
+      </c>
+      <c r="Y20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q2</t>
+        </is>
+      </c>
+      <c r="Z20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q3</t>
+        </is>
+      </c>
+      <c r="AA20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q4</t>
+        </is>
+      </c>
+      <c r="AB20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q5</t>
+        </is>
+      </c>
+      <c r="AC20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q6</t>
+        </is>
+      </c>
+      <c r="AD20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q7</t>
+        </is>
+      </c>
+      <c r="AE20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q8</t>
+        </is>
+      </c>
+      <c r="AF20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q9</t>
+        </is>
+      </c>
+      <c r="AG20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q10</t>
+        </is>
+      </c>
+      <c r="AH20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q11</t>
+        </is>
+      </c>
+      <c r="AI20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q12</t>
+        </is>
+      </c>
+      <c r="AJ20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q13</t>
+        </is>
+      </c>
+      <c r="AK20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q14</t>
+        </is>
+      </c>
+      <c r="AL20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q15</t>
+        </is>
+      </c>
+      <c r="AM20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q16</t>
+        </is>
+      </c>
+      <c r="AN20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q17</t>
+        </is>
+      </c>
+      <c r="AO20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q18</t>
+        </is>
+      </c>
+      <c r="AP20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q19</t>
+        </is>
+      </c>
+      <c r="AQ20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q20</t>
+        </is>
+      </c>
+      <c r="AR20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q21</t>
+        </is>
+      </c>
+      <c r="AS20" s="10" t="inlineStr">
+        <is>
+          <t>G2 Q22</t>
         </is>
       </c>
     </row>
@@ -1969,6 +2665,30 @@
       <c r="S21" s="27" t="n"/>
       <c r="T21" s="27" t="n"/>
       <c r="U21" s="27" t="n"/>
+      <c r="V21" s="27" t="n"/>
+      <c r="W21" s="27" t="n"/>
+      <c r="X21" s="27" t="n"/>
+      <c r="Y21" s="27" t="n"/>
+      <c r="Z21" s="27" t="n"/>
+      <c r="AA21" s="27" t="n"/>
+      <c r="AB21" s="27" t="n"/>
+      <c r="AC21" s="27" t="n"/>
+      <c r="AD21" s="27" t="n"/>
+      <c r="AE21" s="27" t="n"/>
+      <c r="AF21" s="27" t="n"/>
+      <c r="AG21" s="27" t="n"/>
+      <c r="AH21" s="27" t="n"/>
+      <c r="AI21" s="27" t="n"/>
+      <c r="AJ21" s="27" t="n"/>
+      <c r="AK21" s="27" t="n"/>
+      <c r="AL21" s="27" t="n"/>
+      <c r="AM21" s="27" t="n"/>
+      <c r="AN21" s="27" t="n"/>
+      <c r="AO21" s="27" t="n"/>
+      <c r="AP21" s="27" t="n"/>
+      <c r="AQ21" s="27" t="n"/>
+      <c r="AR21" s="27" t="n"/>
+      <c r="AS21" s="27" t="n"/>
     </row>
     <row r="22" ht="33" customHeight="1">
       <c r="A22" s="12" t="n">
@@ -1994,6 +2714,30 @@
       <c r="S22" s="27" t="n"/>
       <c r="T22" s="27" t="n"/>
       <c r="U22" s="27" t="n"/>
+      <c r="V22" s="27" t="n"/>
+      <c r="W22" s="27" t="n"/>
+      <c r="X22" s="27" t="n"/>
+      <c r="Y22" s="27" t="n"/>
+      <c r="Z22" s="27" t="n"/>
+      <c r="AA22" s="27" t="n"/>
+      <c r="AB22" s="27" t="n"/>
+      <c r="AC22" s="27" t="n"/>
+      <c r="AD22" s="27" t="n"/>
+      <c r="AE22" s="27" t="n"/>
+      <c r="AF22" s="27" t="n"/>
+      <c r="AG22" s="27" t="n"/>
+      <c r="AH22" s="27" t="n"/>
+      <c r="AI22" s="27" t="n"/>
+      <c r="AJ22" s="27" t="n"/>
+      <c r="AK22" s="27" t="n"/>
+      <c r="AL22" s="27" t="n"/>
+      <c r="AM22" s="27" t="n"/>
+      <c r="AN22" s="27" t="n"/>
+      <c r="AO22" s="27" t="n"/>
+      <c r="AP22" s="27" t="n"/>
+      <c r="AQ22" s="27" t="n"/>
+      <c r="AR22" s="27" t="n"/>
+      <c r="AS22" s="27" t="n"/>
     </row>
     <row r="23" ht="33" customHeight="1">
       <c r="A23" s="12" t="n">
@@ -2019,6 +2763,30 @@
       <c r="S23" s="27" t="n"/>
       <c r="T23" s="27" t="n"/>
       <c r="U23" s="27" t="n"/>
+      <c r="V23" s="27" t="n"/>
+      <c r="W23" s="27" t="n"/>
+      <c r="X23" s="27" t="n"/>
+      <c r="Y23" s="27" t="n"/>
+      <c r="Z23" s="27" t="n"/>
+      <c r="AA23" s="27" t="n"/>
+      <c r="AB23" s="27" t="n"/>
+      <c r="AC23" s="27" t="n"/>
+      <c r="AD23" s="27" t="n"/>
+      <c r="AE23" s="27" t="n"/>
+      <c r="AF23" s="27" t="n"/>
+      <c r="AG23" s="27" t="n"/>
+      <c r="AH23" s="27" t="n"/>
+      <c r="AI23" s="27" t="n"/>
+      <c r="AJ23" s="27" t="n"/>
+      <c r="AK23" s="27" t="n"/>
+      <c r="AL23" s="27" t="n"/>
+      <c r="AM23" s="27" t="n"/>
+      <c r="AN23" s="27" t="n"/>
+      <c r="AO23" s="27" t="n"/>
+      <c r="AP23" s="27" t="n"/>
+      <c r="AQ23" s="27" t="n"/>
+      <c r="AR23" s="27" t="n"/>
+      <c r="AS23" s="27" t="n"/>
     </row>
     <row r="24" ht="33" customHeight="1">
       <c r="A24" s="12" t="n">
@@ -2044,6 +2812,30 @@
       <c r="S24" s="27" t="n"/>
       <c r="T24" s="27" t="n"/>
       <c r="U24" s="27" t="n"/>
+      <c r="V24" s="27" t="n"/>
+      <c r="W24" s="27" t="n"/>
+      <c r="X24" s="27" t="n"/>
+      <c r="Y24" s="27" t="n"/>
+      <c r="Z24" s="27" t="n"/>
+      <c r="AA24" s="27" t="n"/>
+      <c r="AB24" s="27" t="n"/>
+      <c r="AC24" s="27" t="n"/>
+      <c r="AD24" s="27" t="n"/>
+      <c r="AE24" s="27" t="n"/>
+      <c r="AF24" s="27" t="n"/>
+      <c r="AG24" s="27" t="n"/>
+      <c r="AH24" s="27" t="n"/>
+      <c r="AI24" s="27" t="n"/>
+      <c r="AJ24" s="27" t="n"/>
+      <c r="AK24" s="27" t="n"/>
+      <c r="AL24" s="27" t="n"/>
+      <c r="AM24" s="27" t="n"/>
+      <c r="AN24" s="27" t="n"/>
+      <c r="AO24" s="27" t="n"/>
+      <c r="AP24" s="27" t="n"/>
+      <c r="AQ24" s="27" t="n"/>
+      <c r="AR24" s="27" t="n"/>
+      <c r="AS24" s="27" t="n"/>
     </row>
     <row r="25" ht="33" customHeight="1">
       <c r="A25" s="12" t="n">
@@ -2069,6 +2861,30 @@
       <c r="S25" s="27" t="n"/>
       <c r="T25" s="27" t="n"/>
       <c r="U25" s="27" t="n"/>
+      <c r="V25" s="27" t="n"/>
+      <c r="W25" s="27" t="n"/>
+      <c r="X25" s="27" t="n"/>
+      <c r="Y25" s="27" t="n"/>
+      <c r="Z25" s="27" t="n"/>
+      <c r="AA25" s="27" t="n"/>
+      <c r="AB25" s="27" t="n"/>
+      <c r="AC25" s="27" t="n"/>
+      <c r="AD25" s="27" t="n"/>
+      <c r="AE25" s="27" t="n"/>
+      <c r="AF25" s="27" t="n"/>
+      <c r="AG25" s="27" t="n"/>
+      <c r="AH25" s="27" t="n"/>
+      <c r="AI25" s="27" t="n"/>
+      <c r="AJ25" s="27" t="n"/>
+      <c r="AK25" s="27" t="n"/>
+      <c r="AL25" s="27" t="n"/>
+      <c r="AM25" s="27" t="n"/>
+      <c r="AN25" s="27" t="n"/>
+      <c r="AO25" s="27" t="n"/>
+      <c r="AP25" s="27" t="n"/>
+      <c r="AQ25" s="27" t="n"/>
+      <c r="AR25" s="27" t="n"/>
+      <c r="AS25" s="27" t="n"/>
     </row>
     <row r="26" ht="33" customHeight="1">
       <c r="A26" s="15" t="n">
@@ -2094,6 +2910,30 @@
       <c r="S26" s="28" t="n"/>
       <c r="T26" s="28" t="n"/>
       <c r="U26" s="28" t="n"/>
+      <c r="V26" s="28" t="n"/>
+      <c r="W26" s="28" t="n"/>
+      <c r="X26" s="28" t="n"/>
+      <c r="Y26" s="28" t="n"/>
+      <c r="Z26" s="28" t="n"/>
+      <c r="AA26" s="28" t="n"/>
+      <c r="AB26" s="28" t="n"/>
+      <c r="AC26" s="28" t="n"/>
+      <c r="AD26" s="28" t="n"/>
+      <c r="AE26" s="28" t="n"/>
+      <c r="AF26" s="28" t="n"/>
+      <c r="AG26" s="28" t="n"/>
+      <c r="AH26" s="28" t="n"/>
+      <c r="AI26" s="28" t="n"/>
+      <c r="AJ26" s="28" t="n"/>
+      <c r="AK26" s="28" t="n"/>
+      <c r="AL26" s="28" t="n"/>
+      <c r="AM26" s="28" t="n"/>
+      <c r="AN26" s="28" t="n"/>
+      <c r="AO26" s="28" t="n"/>
+      <c r="AP26" s="28" t="n"/>
+      <c r="AQ26" s="28" t="n"/>
+      <c r="AR26" s="28" t="n"/>
+      <c r="AS26" s="28" t="n"/>
     </row>
     <row r="27" ht="33" customHeight="1">
       <c r="A27" s="12" t="n">
@@ -2119,6 +2959,30 @@
       <c r="S27" s="27" t="n"/>
       <c r="T27" s="27" t="n"/>
       <c r="U27" s="27" t="n"/>
+      <c r="V27" s="27" t="n"/>
+      <c r="W27" s="27" t="n"/>
+      <c r="X27" s="27" t="n"/>
+      <c r="Y27" s="27" t="n"/>
+      <c r="Z27" s="27" t="n"/>
+      <c r="AA27" s="27" t="n"/>
+      <c r="AB27" s="27" t="n"/>
+      <c r="AC27" s="27" t="n"/>
+      <c r="AD27" s="27" t="n"/>
+      <c r="AE27" s="27" t="n"/>
+      <c r="AF27" s="27" t="n"/>
+      <c r="AG27" s="27" t="n"/>
+      <c r="AH27" s="27" t="n"/>
+      <c r="AI27" s="27" t="n"/>
+      <c r="AJ27" s="27" t="n"/>
+      <c r="AK27" s="27" t="n"/>
+      <c r="AL27" s="27" t="n"/>
+      <c r="AM27" s="27" t="n"/>
+      <c r="AN27" s="27" t="n"/>
+      <c r="AO27" s="27" t="n"/>
+      <c r="AP27" s="27" t="n"/>
+      <c r="AQ27" s="27" t="n"/>
+      <c r="AR27" s="27" t="n"/>
+      <c r="AS27" s="27" t="n"/>
     </row>
     <row r="28" ht="33" customHeight="1">
       <c r="A28" s="12" t="n">
@@ -2144,6 +3008,30 @@
       <c r="S28" s="27" t="n"/>
       <c r="T28" s="27" t="n"/>
       <c r="U28" s="27" t="n"/>
+      <c r="V28" s="27" t="n"/>
+      <c r="W28" s="27" t="n"/>
+      <c r="X28" s="27" t="n"/>
+      <c r="Y28" s="27" t="n"/>
+      <c r="Z28" s="27" t="n"/>
+      <c r="AA28" s="27" t="n"/>
+      <c r="AB28" s="27" t="n"/>
+      <c r="AC28" s="27" t="n"/>
+      <c r="AD28" s="27" t="n"/>
+      <c r="AE28" s="27" t="n"/>
+      <c r="AF28" s="27" t="n"/>
+      <c r="AG28" s="27" t="n"/>
+      <c r="AH28" s="27" t="n"/>
+      <c r="AI28" s="27" t="n"/>
+      <c r="AJ28" s="27" t="n"/>
+      <c r="AK28" s="27" t="n"/>
+      <c r="AL28" s="27" t="n"/>
+      <c r="AM28" s="27" t="n"/>
+      <c r="AN28" s="27" t="n"/>
+      <c r="AO28" s="27" t="n"/>
+      <c r="AP28" s="27" t="n"/>
+      <c r="AQ28" s="27" t="n"/>
+      <c r="AR28" s="27" t="n"/>
+      <c r="AS28" s="27" t="n"/>
     </row>
     <row r="29" ht="33" customHeight="1">
       <c r="A29" s="12" t="n">
@@ -2169,6 +3057,30 @@
       <c r="S29" s="27" t="n"/>
       <c r="T29" s="27" t="n"/>
       <c r="U29" s="27" t="n"/>
+      <c r="V29" s="27" t="n"/>
+      <c r="W29" s="27" t="n"/>
+      <c r="X29" s="27" t="n"/>
+      <c r="Y29" s="27" t="n"/>
+      <c r="Z29" s="27" t="n"/>
+      <c r="AA29" s="27" t="n"/>
+      <c r="AB29" s="27" t="n"/>
+      <c r="AC29" s="27" t="n"/>
+      <c r="AD29" s="27" t="n"/>
+      <c r="AE29" s="27" t="n"/>
+      <c r="AF29" s="27" t="n"/>
+      <c r="AG29" s="27" t="n"/>
+      <c r="AH29" s="27" t="n"/>
+      <c r="AI29" s="27" t="n"/>
+      <c r="AJ29" s="27" t="n"/>
+      <c r="AK29" s="27" t="n"/>
+      <c r="AL29" s="27" t="n"/>
+      <c r="AM29" s="27" t="n"/>
+      <c r="AN29" s="27" t="n"/>
+      <c r="AO29" s="27" t="n"/>
+      <c r="AP29" s="27" t="n"/>
+      <c r="AQ29" s="27" t="n"/>
+      <c r="AR29" s="27" t="n"/>
+      <c r="AS29" s="27" t="n"/>
     </row>
     <row r="30" ht="33" customHeight="1">
       <c r="A30" s="12" t="n">
@@ -2194,6 +3106,30 @@
       <c r="S30" s="27" t="n"/>
       <c r="T30" s="27" t="n"/>
       <c r="U30" s="27" t="n"/>
+      <c r="V30" s="27" t="n"/>
+      <c r="W30" s="27" t="n"/>
+      <c r="X30" s="27" t="n"/>
+      <c r="Y30" s="27" t="n"/>
+      <c r="Z30" s="27" t="n"/>
+      <c r="AA30" s="27" t="n"/>
+      <c r="AB30" s="27" t="n"/>
+      <c r="AC30" s="27" t="n"/>
+      <c r="AD30" s="27" t="n"/>
+      <c r="AE30" s="27" t="n"/>
+      <c r="AF30" s="27" t="n"/>
+      <c r="AG30" s="27" t="n"/>
+      <c r="AH30" s="27" t="n"/>
+      <c r="AI30" s="27" t="n"/>
+      <c r="AJ30" s="27" t="n"/>
+      <c r="AK30" s="27" t="n"/>
+      <c r="AL30" s="27" t="n"/>
+      <c r="AM30" s="27" t="n"/>
+      <c r="AN30" s="27" t="n"/>
+      <c r="AO30" s="27" t="n"/>
+      <c r="AP30" s="27" t="n"/>
+      <c r="AQ30" s="27" t="n"/>
+      <c r="AR30" s="27" t="n"/>
+      <c r="AS30" s="27" t="n"/>
     </row>
     <row r="31" ht="33" customHeight="1">
       <c r="A31" s="12" t="n">
@@ -2219,6 +3155,30 @@
       <c r="S31" s="27" t="n"/>
       <c r="T31" s="27" t="n"/>
       <c r="U31" s="27" t="n"/>
+      <c r="V31" s="27" t="n"/>
+      <c r="W31" s="27" t="n"/>
+      <c r="X31" s="27" t="n"/>
+      <c r="Y31" s="27" t="n"/>
+      <c r="Z31" s="27" t="n"/>
+      <c r="AA31" s="27" t="n"/>
+      <c r="AB31" s="27" t="n"/>
+      <c r="AC31" s="27" t="n"/>
+      <c r="AD31" s="27" t="n"/>
+      <c r="AE31" s="27" t="n"/>
+      <c r="AF31" s="27" t="n"/>
+      <c r="AG31" s="27" t="n"/>
+      <c r="AH31" s="27" t="n"/>
+      <c r="AI31" s="27" t="n"/>
+      <c r="AJ31" s="27" t="n"/>
+      <c r="AK31" s="27" t="n"/>
+      <c r="AL31" s="27" t="n"/>
+      <c r="AM31" s="27" t="n"/>
+      <c r="AN31" s="27" t="n"/>
+      <c r="AO31" s="27" t="n"/>
+      <c r="AP31" s="27" t="n"/>
+      <c r="AQ31" s="27" t="n"/>
+      <c r="AR31" s="27" t="n"/>
+      <c r="AS31" s="27" t="n"/>
     </row>
     <row r="32" ht="33" customHeight="1">
       <c r="A32" s="12" t="n">
@@ -2244,6 +3204,30 @@
       <c r="S32" s="27" t="n"/>
       <c r="T32" s="27" t="n"/>
       <c r="U32" s="27" t="n"/>
+      <c r="V32" s="27" t="n"/>
+      <c r="W32" s="27" t="n"/>
+      <c r="X32" s="27" t="n"/>
+      <c r="Y32" s="27" t="n"/>
+      <c r="Z32" s="27" t="n"/>
+      <c r="AA32" s="27" t="n"/>
+      <c r="AB32" s="27" t="n"/>
+      <c r="AC32" s="27" t="n"/>
+      <c r="AD32" s="27" t="n"/>
+      <c r="AE32" s="27" t="n"/>
+      <c r="AF32" s="27" t="n"/>
+      <c r="AG32" s="27" t="n"/>
+      <c r="AH32" s="27" t="n"/>
+      <c r="AI32" s="27" t="n"/>
+      <c r="AJ32" s="27" t="n"/>
+      <c r="AK32" s="27" t="n"/>
+      <c r="AL32" s="27" t="n"/>
+      <c r="AM32" s="27" t="n"/>
+      <c r="AN32" s="27" t="n"/>
+      <c r="AO32" s="27" t="n"/>
+      <c r="AP32" s="27" t="n"/>
+      <c r="AQ32" s="27" t="n"/>
+      <c r="AR32" s="27" t="n"/>
+      <c r="AS32" s="27" t="n"/>
     </row>
     <row r="33" ht="33" customHeight="1">
       <c r="A33" s="15" t="n">
@@ -2269,6 +3253,30 @@
       <c r="S33" s="28" t="n"/>
       <c r="T33" s="28" t="n"/>
       <c r="U33" s="28" t="n"/>
+      <c r="V33" s="28" t="n"/>
+      <c r="W33" s="28" t="n"/>
+      <c r="X33" s="28" t="n"/>
+      <c r="Y33" s="28" t="n"/>
+      <c r="Z33" s="28" t="n"/>
+      <c r="AA33" s="28" t="n"/>
+      <c r="AB33" s="28" t="n"/>
+      <c r="AC33" s="28" t="n"/>
+      <c r="AD33" s="28" t="n"/>
+      <c r="AE33" s="28" t="n"/>
+      <c r="AF33" s="28" t="n"/>
+      <c r="AG33" s="28" t="n"/>
+      <c r="AH33" s="28" t="n"/>
+      <c r="AI33" s="28" t="n"/>
+      <c r="AJ33" s="28" t="n"/>
+      <c r="AK33" s="28" t="n"/>
+      <c r="AL33" s="28" t="n"/>
+      <c r="AM33" s="28" t="n"/>
+      <c r="AN33" s="28" t="n"/>
+      <c r="AO33" s="28" t="n"/>
+      <c r="AP33" s="28" t="n"/>
+      <c r="AQ33" s="28" t="n"/>
+      <c r="AR33" s="28" t="n"/>
+      <c r="AS33" s="28" t="n"/>
     </row>
     <row r="34" ht="33" customHeight="1">
       <c r="A34" s="12" t="n">
@@ -2294,6 +3302,30 @@
       <c r="S34" s="27" t="n"/>
       <c r="T34" s="27" t="n"/>
       <c r="U34" s="27" t="n"/>
+      <c r="V34" s="27" t="n"/>
+      <c r="W34" s="27" t="n"/>
+      <c r="X34" s="27" t="n"/>
+      <c r="Y34" s="27" t="n"/>
+      <c r="Z34" s="27" t="n"/>
+      <c r="AA34" s="27" t="n"/>
+      <c r="AB34" s="27" t="n"/>
+      <c r="AC34" s="27" t="n"/>
+      <c r="AD34" s="27" t="n"/>
+      <c r="AE34" s="27" t="n"/>
+      <c r="AF34" s="27" t="n"/>
+      <c r="AG34" s="27" t="n"/>
+      <c r="AH34" s="27" t="n"/>
+      <c r="AI34" s="27" t="n"/>
+      <c r="AJ34" s="27" t="n"/>
+      <c r="AK34" s="27" t="n"/>
+      <c r="AL34" s="27" t="n"/>
+      <c r="AM34" s="27" t="n"/>
+      <c r="AN34" s="27" t="n"/>
+      <c r="AO34" s="27" t="n"/>
+      <c r="AP34" s="27" t="n"/>
+      <c r="AQ34" s="27" t="n"/>
+      <c r="AR34" s="27" t="n"/>
+      <c r="AS34" s="27" t="n"/>
     </row>
     <row r="35" ht="33" customHeight="1" thickBot="1">
       <c r="A35" s="12" t="n">
@@ -2319,6 +3351,30 @@
       <c r="S35" s="27" t="n"/>
       <c r="T35" s="27" t="n"/>
       <c r="U35" s="27" t="n"/>
+      <c r="V35" s="27" t="n"/>
+      <c r="W35" s="27" t="n"/>
+      <c r="X35" s="27" t="n"/>
+      <c r="Y35" s="27" t="n"/>
+      <c r="Z35" s="27" t="n"/>
+      <c r="AA35" s="27" t="n"/>
+      <c r="AB35" s="27" t="n"/>
+      <c r="AC35" s="27" t="n"/>
+      <c r="AD35" s="27" t="n"/>
+      <c r="AE35" s="27" t="n"/>
+      <c r="AF35" s="27" t="n"/>
+      <c r="AG35" s="27" t="n"/>
+      <c r="AH35" s="27" t="n"/>
+      <c r="AI35" s="27" t="n"/>
+      <c r="AJ35" s="27" t="n"/>
+      <c r="AK35" s="27" t="n"/>
+      <c r="AL35" s="27" t="n"/>
+      <c r="AM35" s="27" t="n"/>
+      <c r="AN35" s="27" t="n"/>
+      <c r="AO35" s="27" t="n"/>
+      <c r="AP35" s="27" t="n"/>
+      <c r="AQ35" s="27" t="n"/>
+      <c r="AR35" s="27" t="n"/>
+      <c r="AS35" s="27" t="n"/>
     </row>
     <row r="36" ht="33" customHeight="1"/>
     <row r="37" ht="48.75" customHeight="1"/>
@@ -2336,10 +3392,10 @@
     <row r="55" ht="45" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="T1:U1"/>
-    <mergeCell ref="A1:S1"/>
-    <mergeCell ref="B2:U2"/>
-    <mergeCell ref="B19:U19"/>
+    <mergeCell ref="A1:AP1"/>
+    <mergeCell ref="B2:AS2"/>
+    <mergeCell ref="B19:AS19"/>
+    <mergeCell ref="AQ1:AS1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>